<commit_message>
Table builder removes masses and prm_sensitvities to cal_sensitivites
</commit_message>
<xml_diff>
--- a/Total_Oxide_Calculations/Oxides.xlsx
+++ b/Total_Oxide_Calculations/Oxides.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unibe365-my.sharepoint.com/personal/sebastian_stumpf_unibe_ch/Documents/PhD/ICP-Base/ICP-Base_dev/Total_Oxide_Calculations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_C93881D2F499C0CA9E24614525B7E03D54DD654E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7009A8F-4C0B-49F2-B124-5212A6E450DF}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_C93881D2F499C0CA9E24614525B7E03D54DD654E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEC36185-E875-4A39-AE34-6A92EC20552B}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="159">
   <si>
     <t>SiO2</t>
   </si>
@@ -499,6 +499,9 @@
   </si>
   <si>
     <t>Ni62</t>
+  </si>
+  <si>
+    <t>Sr88</t>
   </si>
 </sst>
 </file>
@@ -840,16 +843,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>136</v>
       </c>
@@ -866,7 +869,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -882,7 +885,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -901,7 +904,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -917,7 +920,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -933,7 +936,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -949,7 +952,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -965,7 +968,7 @@
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -981,7 +984,7 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -997,7 +1000,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1016,7 +1019,7 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1035,7 +1038,7 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1051,7 +1054,7 @@
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1067,7 +1070,7 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
@@ -1086,7 +1089,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -1102,7 +1105,7 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -1121,7 +1124,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -1137,7 +1140,7 @@
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -1153,7 +1156,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -1169,7 +1172,7 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
@@ -1185,7 +1188,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
@@ -1201,7 +1204,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
@@ -1220,7 +1223,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -1236,7 +1239,7 @@
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
@@ -1252,7 +1255,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
@@ -1268,7 +1271,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
@@ -1284,7 +1287,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>37</v>
       </c>
@@ -1300,7 +1303,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>38</v>
       </c>
@@ -1316,7 +1319,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>134</v>
       </c>
@@ -1332,7 +1335,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
@@ -1351,7 +1354,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>40</v>
       </c>
@@ -1367,7 +1370,7 @@
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>41</v>
       </c>
@@ -1383,7 +1386,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>42</v>
       </c>
@@ -1399,7 +1402,7 @@
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>43</v>
       </c>
@@ -1418,7 +1421,7 @@
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>45</v>
       </c>
@@ -1434,7 +1437,7 @@
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>46</v>
       </c>
@@ -1453,7 +1456,7 @@
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>47</v>
       </c>
@@ -1472,7 +1475,7 @@
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>48</v>
       </c>
@@ -1488,7 +1491,7 @@
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>49</v>
       </c>
@@ -1504,7 +1507,7 @@
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>50</v>
       </c>
@@ -1523,7 +1526,7 @@
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>52</v>
       </c>
@@ -1539,7 +1542,7 @@
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>53</v>
       </c>
@@ -1558,7 +1561,7 @@
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>55</v>
       </c>
@@ -1574,7 +1577,7 @@
       <c r="I43" s="3"/>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>57</v>
       </c>
@@ -1590,7 +1593,7 @@
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>58</v>
       </c>
@@ -1606,7 +1609,7 @@
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>59</v>
       </c>
@@ -1622,7 +1625,7 @@
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>60</v>
       </c>
@@ -1638,7 +1641,7 @@
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>61</v>
       </c>
@@ -1654,7 +1657,7 @@
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>62</v>
       </c>
@@ -1673,7 +1676,7 @@
       <c r="I49" s="3"/>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>63</v>
       </c>
@@ -1689,7 +1692,7 @@
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>64</v>
       </c>
@@ -1705,7 +1708,7 @@
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>65</v>
       </c>
@@ -1721,7 +1724,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>66</v>
       </c>
@@ -1740,7 +1743,7 @@
       <c r="I53" s="3"/>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>67</v>
       </c>
@@ -1756,7 +1759,7 @@
       <c r="I54" s="3"/>
       <c r="J54" s="3"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>68</v>
       </c>
@@ -1772,7 +1775,7 @@
       <c r="I55" s="3"/>
       <c r="J55" s="3"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>69</v>
       </c>
@@ -1782,13 +1785,16 @@
       <c r="C56" s="1">
         <v>1.1826000000000001</v>
       </c>
+      <c r="D56" t="s">
+        <v>158</v>
+      </c>
       <c r="E56" s="1" t="s">
         <v>155</v>
       </c>
       <c r="I56" s="3"/>
       <c r="J56" s="3"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>71</v>
       </c>
@@ -1804,7 +1810,7 @@
       <c r="I57" s="3"/>
       <c r="J57" s="3"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>72</v>
       </c>
@@ -1820,7 +1826,7 @@
       <c r="I58" s="3"/>
       <c r="J58" s="3"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>73</v>
       </c>
@@ -1836,7 +1842,7 @@
       <c r="I59" s="3"/>
       <c r="J59" s="3"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>74</v>
       </c>
@@ -1852,7 +1858,7 @@
       <c r="I60" s="3"/>
       <c r="J60" s="3"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>75</v>
       </c>
@@ -1871,7 +1877,7 @@
       <c r="I61" s="3"/>
       <c r="J61" s="3"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>76</v>
       </c>
@@ -1887,7 +1893,7 @@
       <c r="I62" s="3"/>
       <c r="J62" s="3"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>77</v>
       </c>
@@ -1903,7 +1909,7 @@
       <c r="I63" s="3"/>
       <c r="J63" s="3"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>78</v>
       </c>
@@ -1919,7 +1925,7 @@
       <c r="I64" s="3"/>
       <c r="J64" s="3"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>79</v>
       </c>
@@ -1935,7 +1941,7 @@
       <c r="I65" s="3"/>
       <c r="J65" s="3"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>80</v>
       </c>
@@ -1951,7 +1957,7 @@
       <c r="I66" s="3"/>
       <c r="J66" s="3"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>81</v>
       </c>
@@ -1967,7 +1973,7 @@
       <c r="I67" s="3"/>
       <c r="J67" s="3"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>82</v>
       </c>
@@ -1983,7 +1989,7 @@
       <c r="I68" s="3"/>
       <c r="J68" s="3"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>83</v>
       </c>
@@ -1999,7 +2005,7 @@
       <c r="I69" s="3"/>
       <c r="J69" s="3"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>85</v>
       </c>
@@ -2015,40 +2021,40 @@
       <c r="I70" s="3"/>
       <c r="J70" s="3"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F83" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New RM files, updated manuals, fixed small bug in moving average
</commit_message>
<xml_diff>
--- a/Total_Oxide_Calculations/Oxides.xlsx
+++ b/Total_Oxide_Calculations/Oxides.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unibe365-my.sharepoint.com/personal/sebastian_stumpf_unibe_ch/Documents/PhD/ICP-Base/ICP-Base_dev/Total_Oxide_Calculations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_C93881D2F499C0CA9E24614525B7E03D54DD654E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A378CB5A-9121-478E-99AD-DE9287471768}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_C93881D2F499C0CA9E24614525B7E03D54DD654E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9650F2A-7051-4E97-A306-B6FB9AEFC7A1}"/>
   <bookViews>
-    <workbookView xWindow="28860" yWindow="195" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -521,18 +521,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -547,7 +541,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -557,10 +551,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -876,7 +867,7 @@
       <c r="B2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="4">
         <v>1.0742</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -892,8 +883,8 @@
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1">
-        <v>1.8895</v>
+      <c r="C3" s="4">
+        <v>1.8894</v>
       </c>
       <c r="D3" t="s">
         <v>145</v>
@@ -911,8 +902,8 @@
       <c r="B4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="5">
-        <v>1.32</v>
+      <c r="C4" s="4">
+        <v>1.3203</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>154</v>
@@ -927,7 +918,7 @@
       <c r="B5" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="4">
         <v>1.1217999999999999</v>
       </c>
       <c r="E5" s="1" t="s">
@@ -943,8 +934,8 @@
       <c r="B6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="1">
-        <v>3.2202000000000002</v>
+      <c r="C6" s="4">
+        <v>3.22</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>154</v>
@@ -959,7 +950,7 @@
       <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="4">
         <v>1.1165</v>
       </c>
       <c r="E7" s="1" t="s">
@@ -975,7 +966,7 @@
       <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="4">
         <v>2.7753000000000001</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -991,7 +982,7 @@
       <c r="B9" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="4">
         <v>1.1148</v>
       </c>
       <c r="E9" s="1" t="s">
@@ -1007,7 +998,7 @@
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="4">
         <v>1</v>
       </c>
       <c r="D10" t="s">
@@ -1026,7 +1017,7 @@
       <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="4">
         <v>1.3992</v>
       </c>
       <c r="D11" t="s">
@@ -1045,7 +1036,7 @@
       <c r="B12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="4">
         <v>1.1423000000000001</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1061,7 +1052,7 @@
       <c r="B13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="4">
         <v>1.2283999999999999</v>
       </c>
       <c r="E13" s="1" t="s">
@@ -1077,7 +1068,7 @@
       <c r="B14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="4">
         <v>1</v>
       </c>
       <c r="D14" t="s">
@@ -1096,7 +1087,7 @@
       <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="4">
         <v>1.2715000000000001</v>
       </c>
       <c r="E15" s="1" t="s">
@@ -1112,8 +1103,8 @@
       <c r="B16" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="1">
-        <v>1.4616</v>
+      <c r="C16" s="4">
+        <v>1.4615</v>
       </c>
       <c r="D16" t="s">
         <v>149</v>
@@ -1131,8 +1122,8 @@
       <c r="B17" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="5">
-        <v>1.0629999999999999</v>
+      <c r="C17" s="4">
+        <v>1.0602</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>154</v>
@@ -1147,7 +1138,7 @@
       <c r="B18" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="4">
         <v>1.2518</v>
       </c>
       <c r="E18" s="1" t="s">
@@ -1163,8 +1154,8 @@
       <c r="B19" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C19" s="5">
-        <v>1.1479999999999999</v>
+      <c r="C19" s="4">
+        <v>1.1476999999999999</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>154</v>
@@ -1179,8 +1170,8 @@
       <c r="B20" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C20" s="5">
-        <v>1.143</v>
+      <c r="C20" s="4">
+        <v>1.1435</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>154</v>
@@ -1195,8 +1186,8 @@
       <c r="B21" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="5">
-        <v>1.1579999999999999</v>
+      <c r="C21" s="4">
+        <v>1.1578999999999999</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>154</v>
@@ -1211,7 +1202,7 @@
       <c r="B22" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="4">
         <v>1.2865</v>
       </c>
       <c r="D22" t="s">
@@ -1230,7 +1221,7 @@
       <c r="B23" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="4">
         <v>1.3442000000000001</v>
       </c>
       <c r="E23" s="1" t="s">
@@ -1247,7 +1238,7 @@
         <v>98</v>
       </c>
       <c r="C24" s="4">
-        <v>1.152604887044721</v>
+        <v>1.1526000000000001</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>154</v>
@@ -1262,8 +1253,8 @@
       <c r="B25" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="1">
-        <v>1.4408000000000001</v>
+      <c r="C25" s="4">
+        <v>1.4406000000000001</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>154</v>
@@ -1278,8 +1269,8 @@
       <c r="B26" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="5">
-        <v>1.2110000000000001</v>
+      <c r="C26" s="4">
+        <v>1.1793</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>154</v>
@@ -1294,8 +1285,8 @@
       <c r="B27" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="5">
-        <v>1.1459999999999999</v>
+      <c r="C27" s="4">
+        <v>1.1455</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>154</v>
@@ -1310,8 +1301,8 @@
       <c r="B28" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C28" s="5">
-        <v>1.2030000000000001</v>
+      <c r="C28" s="4">
+        <v>1.2090000000000001</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>154</v>
@@ -1326,7 +1317,7 @@
       <c r="B29" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="4">
         <v>1.1665000000000001</v>
       </c>
       <c r="E29" s="1" t="s">
@@ -1342,7 +1333,7 @@
       <c r="B30" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="4">
         <v>1.2045999999999999</v>
       </c>
       <c r="D30" t="s">
@@ -1361,7 +1352,7 @@
       <c r="B31" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="4">
         <v>1.1728000000000001</v>
       </c>
       <c r="E31" s="1" t="s">
@@ -1377,8 +1368,8 @@
       <c r="B32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="1">
-        <v>2.1528999999999998</v>
+      <c r="C32" s="4">
+        <v>2.1427999999999998</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>154</v>
@@ -1393,8 +1384,8 @@
       <c r="B33" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C33" s="5">
-        <v>1.137</v>
+      <c r="C33" s="4">
+        <v>1.1372</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>154</v>
@@ -1409,7 +1400,7 @@
       <c r="B34" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" s="4">
         <v>1.6583000000000001</v>
       </c>
       <c r="D34" t="s">
@@ -1428,7 +1419,7 @@
       <c r="B35" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C35" s="4">
         <v>1.2911999999999999</v>
       </c>
       <c r="E35" s="1" t="s">
@@ -1444,8 +1435,8 @@
       <c r="B36" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C36" s="5">
-        <v>1.5</v>
+      <c r="C36" s="4">
+        <v>1.5002</v>
       </c>
       <c r="D36" t="s">
         <v>143</v>
@@ -1463,7 +1454,7 @@
       <c r="B37" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="4">
         <v>1.3480000000000001</v>
       </c>
       <c r="D37" t="s">
@@ -1482,8 +1473,8 @@
       <c r="B38" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C38" s="5">
-        <v>1.431</v>
+      <c r="C38" s="4">
+        <v>1.4305000000000001</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>154</v>
@@ -1498,8 +1489,8 @@
       <c r="B39" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C39" s="5">
-        <v>1.1659999999999999</v>
+      <c r="C39" s="4">
+        <v>1.1664000000000001</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>154</v>
@@ -1514,7 +1505,7 @@
       <c r="B40" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C40" s="1">
+      <c r="C40" s="4">
         <v>1.2726</v>
       </c>
       <c r="D40" t="s">
@@ -1533,8 +1524,8 @@
       <c r="B41" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C41" s="1">
-        <v>2.2913999999999999</v>
+      <c r="C41" s="4">
+        <v>2.2913000000000001</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>154</v>
@@ -1549,8 +1540,8 @@
       <c r="B42" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="1">
-        <v>1.0771999999999999</v>
+      <c r="C42" s="4">
+        <v>1.0772999999999999</v>
       </c>
       <c r="D42" t="s">
         <v>155</v>
@@ -1568,8 +1559,8 @@
       <c r="B43" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C43" s="5">
-        <v>1.206</v>
+      <c r="C43" s="4">
+        <v>1.1503000000000001</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>154</v>
@@ -1584,8 +1575,8 @@
       <c r="B44" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C44" s="5">
-        <v>1.208</v>
+      <c r="C44" s="4">
+        <v>1.1702999999999999</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>154</v>
@@ -1600,8 +1591,8 @@
       <c r="B45" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C45" s="5">
-        <v>1.2130000000000001</v>
+      <c r="C45" s="4">
+        <v>1.1639999999999999</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>154</v>
@@ -1616,7 +1607,7 @@
       <c r="B46" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C46" s="1">
+      <c r="C46" s="4">
         <v>1.0935999999999999</v>
       </c>
       <c r="E46" s="1" t="s">
@@ -1632,8 +1623,8 @@
       <c r="B47" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C47" s="5">
-        <v>1.881</v>
+      <c r="C47" s="4">
+        <v>1.3007</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>154</v>
@@ -1648,8 +1639,8 @@
       <c r="B48" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C48" s="5">
-        <v>1.3660000000000001</v>
+      <c r="C48" s="4">
+        <v>1.2332000000000001</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>154</v>
@@ -1664,8 +1655,8 @@
       <c r="B49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C49" s="5">
-        <v>2.4980000000000002</v>
+      <c r="C49" s="4">
+        <v>2.4965999999999999</v>
       </c>
       <c r="D49" t="s">
         <v>150</v>
@@ -1683,7 +1674,7 @@
       <c r="B50" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C50" s="1">
+      <c r="C50" s="4">
         <v>1.1971000000000001</v>
       </c>
       <c r="E50" s="1" t="s">
@@ -1699,8 +1690,8 @@
       <c r="B51" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C51" s="5">
-        <v>1.546</v>
+      <c r="C51" s="4">
+        <v>1.5338000000000001</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>154</v>
@@ -1715,8 +1706,8 @@
       <c r="B52" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C52" s="5">
-        <v>1.3660000000000001</v>
+      <c r="C52" s="4">
+        <v>1.4052</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>154</v>
@@ -1731,7 +1722,7 @@
       <c r="B53" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C53" s="1">
+      <c r="C53" s="4">
         <v>2.1393</v>
       </c>
       <c r="D53" t="s">
@@ -1750,8 +1741,8 @@
       <c r="B54" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C54" s="5">
-        <v>1.1599999999999999</v>
+      <c r="C54" s="4">
+        <v>1.1596</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>154</v>
@@ -1766,7 +1757,7 @@
       <c r="B55" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C55" s="1">
+      <c r="C55" s="4">
         <v>1.2695000000000001</v>
       </c>
       <c r="E55" s="1" t="s">
@@ -1782,7 +1773,7 @@
       <c r="B56" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C56" s="1">
+      <c r="C56" s="4">
         <v>1.1826000000000001</v>
       </c>
       <c r="D56" t="s">
@@ -1801,8 +1792,8 @@
       <c r="B57" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C57" s="1">
-        <v>1.2211000000000001</v>
+      <c r="C57" s="4">
+        <v>1.2210000000000001</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>154</v>
@@ -1817,8 +1808,8 @@
       <c r="B58" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="5">
-        <v>1.1759999999999999</v>
+      <c r="C58" s="4">
+        <v>1.151</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>154</v>
@@ -1833,7 +1824,7 @@
       <c r="B59" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C59" s="1">
+      <c r="C59" s="4">
         <v>1.2507999999999999</v>
       </c>
       <c r="E59" s="1" t="s">
@@ -1849,8 +1840,8 @@
       <c r="B60" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C60" s="5">
-        <v>1.137</v>
+      <c r="C60" s="4">
+        <v>1.1378999999999999</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>154</v>
@@ -1865,8 +1856,8 @@
       <c r="B61" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C61" s="5">
-        <v>1.6679999999999999</v>
+      <c r="C61" s="4">
+        <v>1.6685000000000001</v>
       </c>
       <c r="D61" t="s">
         <v>147</v>
@@ -1884,8 +1875,8 @@
       <c r="B62" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C62" s="5">
-        <v>1.123</v>
+      <c r="C62" s="4">
+        <v>1.1173999999999999</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>154</v>
@@ -1900,8 +1891,8 @@
       <c r="B63" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="5">
-        <v>1.1419999999999999</v>
+      <c r="C63" s="4">
+        <v>1.1420999999999999</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>154</v>
@@ -1916,7 +1907,7 @@
       <c r="B64" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C64" s="1">
+      <c r="C64" s="4">
         <v>1.1344000000000001</v>
       </c>
       <c r="E64" s="1" t="s">
@@ -1932,7 +1923,7 @@
       <c r="B65" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C65" s="1">
+      <c r="C65" s="4">
         <v>1.7851999999999999</v>
       </c>
       <c r="E65" s="1" t="s">
@@ -1948,8 +1939,8 @@
       <c r="B66" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C66" s="5">
-        <v>1.2609999999999999</v>
+      <c r="C66" s="4">
+        <v>1.2611000000000001</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>154</v>
@@ -1964,8 +1955,8 @@
       <c r="B67" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C67" s="5">
-        <v>1.2789999999999999</v>
+      <c r="C67" s="4">
+        <v>1.2699</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>154</v>
@@ -1980,8 +1971,8 @@
       <c r="B68" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C68" s="5">
-        <v>1.139</v>
+      <c r="C68" s="4">
+        <v>1.1387</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>154</v>
@@ -1996,8 +1987,8 @@
       <c r="B69" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C69" s="1">
-        <v>1.2446999999999999</v>
+      <c r="C69" s="4">
+        <v>1.2445999999999999</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>154</v>
@@ -2012,7 +2003,7 @@
       <c r="B70" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C70" s="1">
+      <c r="C70" s="4">
         <v>1.3508</v>
       </c>
       <c r="E70" s="1" t="s">

</xml_diff>